<commit_message>
feat: cap nhat nhan vien Vo Thi Hang vao bao cao theo target T10 (18 BHX + 2 GS25, target 1,007,529,600d)
</commit_message>
<xml_diff>
--- a/Team_CamGiang_Report.xlsx
+++ b/Team_CamGiang_Report.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tiến độ Team" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Chi tiết CVS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Data BHX" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Config" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Chi tiết SKU FamilyMart" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ Team" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chi tiết CVS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data BHX" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chi tiết SKU FamilyMart" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Chi tiết SKU FamilyMart'!$A$5:$BB$40</definedName>
@@ -391,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -695,6 +695,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1098,7 +1101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H22"/>
+  <dimension ref="A2:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1193,20 +1196,23 @@
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
+      <c r="A7" t="n">
+        <v>11833869329</v>
+      </c>
       <c r="B7" s="12" t="n">
-        <v>10826339729</v>
+        <v>3911111125</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>3551927443</v>
+        <v>359247028</v>
       </c>
       <c r="D7" s="12" t="n">
-        <v>359247028</v>
+        <v>4270358153</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>3911174471</v>
+        <v>7563511176</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>6915165258</v>
+        <v>0.360858991617821</v>
       </c>
       <c r="G7" s="14" t="n">
         <v>0.3612647089323572</v>
@@ -1513,6 +1519,32 @@
         <v>0.2853565874090838</v>
       </c>
     </row>
+    <row r="23">
+      <c r="B23" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>Võ Thị Hằng</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="n">
+        <v>1007529600</v>
+      </c>
+      <c r="E23" s="19" t="n">
+        <v>359183682</v>
+      </c>
+      <c r="F23" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="19" t="n">
+        <v>359183682</v>
+      </c>
+      <c r="H23" s="20" t="n">
+        <v>0.3564993842364532</v>
+      </c>
+    </row>
+    <row r="24"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B5:H5"/>
@@ -1542,7 +1574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:M20"/>
+  <dimension ref="A2:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2070,62 +2102,103 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="30" t="n"/>
-      <c r="C17" s="31" t="inlineStr">
+      <c r="B17" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>Võ Thị Hằng</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="n">
+        <v>1007529600</v>
+      </c>
+      <c r="E17" s="27" t="n">
+        <v>359183682</v>
+      </c>
+      <c r="F17" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="28" t="n">
+        <v>359183682</v>
+      </c>
+      <c r="M17" s="29" t="n">
+        <v>0.3564993842364532</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="30" t="n"/>
+      <c r="C18" s="31" t="inlineStr">
         <is>
           <t>TỔNG TEAM</t>
         </is>
       </c>
-      <c r="D17" s="32">
-        <f>SUM(D7:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="32">
-        <f>SUM(E7:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="32">
-        <f>SUM(F7:F16)</f>
-        <v/>
-      </c>
-      <c r="G17" s="32">
-        <f>SUM(G7:G16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="32">
-        <f>SUM(H7:H16)</f>
-        <v/>
-      </c>
-      <c r="I17" s="32">
-        <f>SUM(I7:I16)</f>
-        <v/>
-      </c>
-      <c r="J17" s="32">
-        <f>SUM(J7:J16)</f>
-        <v/>
-      </c>
-      <c r="K17" s="32">
-        <f>SUM(K7:K16)</f>
-        <v/>
-      </c>
-      <c r="L17" s="32">
-        <f>SUM(L7:L16)</f>
-        <v/>
-      </c>
-      <c r="M17" s="33">
-        <f>L17/D17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="34" t="inlineStr">
+      <c r="D18" s="32">
+        <f>SUM(D7:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="32">
+        <f>SUM(E7:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="32">
+        <f>SUM(F7:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="32">
+        <f>SUM(G7:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="32">
+        <f>SUM(H7:H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="32">
+        <f>SUM(I7:I17)</f>
+        <v/>
+      </c>
+      <c r="J18" s="32">
+        <f>SUM(J7:J17)</f>
+        <v/>
+      </c>
+      <c r="K18" s="32">
+        <f>SUM(K7:K17)</f>
+        <v/>
+      </c>
+      <c r="L18" s="32">
+        <f>SUM(L7:L17)</f>
+        <v/>
+      </c>
+      <c r="M18" s="33">
+        <f>L18/D18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="B20" s="34" t="inlineStr">
         <is>
           <t>📌 % Đạt ≥ % Timegone (46.7%) → Vượt/Đạt tiến độ 🟢 (#28E11F) | Cận Timegone (35.0% - &lt;46.7%) → Cảnh báo 🟠 (#F5991F) | Thấp hơn nhiều (&lt;35.0%) → Cần đẩy nhanh 🔴 (#DD2323)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="35" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="35" t="inlineStr">
         <is>
           <t>🧮 BHX cố định = (Tổng BHX ÷ 232) × Số CH phụ trách | Thực Hiện = BHX + GS25 + 7E + FM + CK + HĐ + WMP | % Đạt = TH ÷ Target</t>
         </is>
@@ -2161,7 +2234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F163"/>
+  <dimension ref="A1:F166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5179,21 +5252,6 @@
       <c r="A119" s="39" t="n">
         <v>103</v>
       </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>Nguyễn Thị Thanh Thủy</t>
-        </is>
-      </c>
-      <c r="C119" s="44" t="inlineStr">
-        <is>
-          <t>Circle K</t>
-        </is>
-      </c>
-      <c r="D119" s="41" t="inlineStr">
-        <is>
-          <t>CVS_CIRCLEK.79.4260</t>
-        </is>
-      </c>
       <c r="E119" s="41" t="inlineStr">
         <is>
           <t>117/21, Thùy Vân, P.Vũng Tàu, TP.Hồ Chí Minh</t>
@@ -6214,19 +6272,89 @@
     </row>
     <row r="158"/>
     <row r="159">
-      <c r="A159" s="49" t="inlineStr">
+      <c r="A159" s="36" t="inlineStr">
+        <is>
+          <t>👤 Võ Thị Hằng (2 cửa hàng CVS)</t>
+        </is>
+      </c>
+      <c r="E159" s="37" t="inlineStr">
+        <is>
+          <t>TỔNG CVS:</t>
+        </is>
+      </c>
+      <c r="F159" s="109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="39" t="n">
+        <v>139</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Võ Thị Hằng</t>
+        </is>
+      </c>
+      <c r="C160" s="48" t="inlineStr">
+        <is>
+          <t>GS25</t>
+        </is>
+      </c>
+      <c r="D160" s="41" t="inlineStr">
+        <is>
+          <t>CVS_GS25.75.6976</t>
+        </is>
+      </c>
+      <c r="E160" s="41" t="inlineStr">
+        <is>
+          <t>GS25 Lê Duẩn - Long Thành</t>
+        </is>
+      </c>
+      <c r="F160" s="42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="39" t="n">
+        <v>140</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Võ Thị Hằng</t>
+        </is>
+      </c>
+      <c r="C161" s="48" t="inlineStr">
+        <is>
+          <t>GS25</t>
+        </is>
+      </c>
+      <c r="D161" s="41" t="inlineStr">
+        <is>
+          <t>CVS_GS25.75.6975</t>
+        </is>
+      </c>
+      <c r="E161" s="41" t="inlineStr">
+        <is>
+          <t>Siêu thị GS-25 35, Nguyễn Đình Chiểu</t>
+        </is>
+      </c>
+      <c r="F161" s="42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="49" t="inlineStr">
         <is>
           <t>🎯 TỔNG CVS TOÀN TEAM</t>
         </is>
       </c>
-      <c r="F159" s="50" t="n">
+      <c r="F163" s="50" t="n">
         <v>372666880</v>
       </c>
     </row>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A159:D159"/>
@@ -6697,7 +6825,7 @@
         </is>
       </c>
       <c r="B10" s="61" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -6707,7 +6835,7 @@
         </is>
       </c>
       <c r="B11" s="61" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
feat: cap nhat 11 nhan vien (Vo Thi Hang) va bang chi tieu Target T10/2026 tren toan bo he thong
</commit_message>
<xml_diff>
--- a/Team_CamGiang_Report.xlsx
+++ b/Team_CamGiang_Report.xlsx
@@ -1101,7 +1101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H24"/>
+  <dimension ref="A2:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1197,7 +1197,7 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" t="n">
-        <v>11833869329</v>
+        <v>12299713233</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>3911111125</v>
@@ -1279,7 +1279,7 @@
         </is>
       </c>
       <c r="D13" s="19" t="n">
-        <v>1346491228</v>
+        <v>1427158977</v>
       </c>
       <c r="E13" s="19" t="n">
         <v>498866214</v>
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="D14" s="19" t="n">
-        <v>1292631579</v>
+        <v>1490030916</v>
       </c>
       <c r="E14" s="19" t="n">
         <v>478911565</v>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="D15" s="19" t="n">
-        <v>1354847566</v>
+        <v>1553803206</v>
       </c>
       <c r="E15" s="19" t="n">
         <v>498866214</v>
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="D16" s="19" t="n">
-        <v>1399499656</v>
+        <v>1439209643</v>
       </c>
       <c r="E16" s="19" t="n">
         <v>498866214</v>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="D17" s="19" t="n">
-        <v>1181190660</v>
+        <v>1224747376</v>
       </c>
       <c r="E17" s="19" t="n">
         <v>419047620</v>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="D18" s="19" t="n">
-        <v>1240952244</v>
+        <v>1347067397</v>
       </c>
       <c r="E18" s="19" t="n">
         <v>419047620</v>
@@ -1429,7 +1429,7 @@
         </is>
       </c>
       <c r="D19" s="19" t="n">
-        <v>583256268</v>
+        <v>543282274</v>
       </c>
       <c r="E19" s="19" t="n">
         <v>119727891</v>
@@ -1454,7 +1454,7 @@
         </is>
       </c>
       <c r="D20" s="19" t="n">
-        <v>1161621042</v>
+        <v>1230123482</v>
       </c>
       <c r="E20" s="19" t="n">
         <v>399092971</v>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="D21" s="19" t="n">
-        <v>864811602</v>
+        <v>735943613</v>
       </c>
       <c r="E21" s="19" t="n">
         <v>219501134</v>
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="D22" s="19" t="n">
-        <v>401037884</v>
+        <v>300816749</v>
       </c>
       <c r="E22" s="19" t="n">
         <v>0</v>
@@ -1544,7 +1544,6 @@
         <v>0.3564993842364532</v>
       </c>
     </row>
-    <row r="24"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B5:H5"/>
@@ -1574,7 +1573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:M21"/>
+  <dimension ref="B2:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1711,7 +1710,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>1181190660</v>
+        <v>1224747376</v>
       </c>
       <c r="E7" s="27" t="n">
         <v>419047620</v>
@@ -1751,7 +1750,7 @@
         </is>
       </c>
       <c r="D8" s="27" t="n">
-        <v>1354847566</v>
+        <v>1553803206</v>
       </c>
       <c r="E8" s="27" t="n">
         <v>498866214</v>
@@ -1791,7 +1790,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>1399499656</v>
+        <v>1439209643</v>
       </c>
       <c r="E9" s="27" t="n">
         <v>498866214</v>
@@ -1831,7 +1830,7 @@
         </is>
       </c>
       <c r="D10" s="27" t="n">
-        <v>1240952244</v>
+        <v>1347067397</v>
       </c>
       <c r="E10" s="27" t="n">
         <v>419047620</v>
@@ -1871,7 +1870,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>1292631579</v>
+        <v>1490030916</v>
       </c>
       <c r="E11" s="27" t="n">
         <v>478911565</v>
@@ -1911,7 +1910,7 @@
         </is>
       </c>
       <c r="D12" s="27" t="n">
-        <v>864811602</v>
+        <v>735943613</v>
       </c>
       <c r="E12" s="27" t="n">
         <v>219501134</v>
@@ -1951,7 +1950,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>401037884</v>
+        <v>300816749</v>
       </c>
       <c r="E13" s="27" t="n">
         <v>0</v>
@@ -1991,7 +1990,7 @@
         </is>
       </c>
       <c r="D14" s="27" t="n">
-        <v>1346491228</v>
+        <v>1427158977</v>
       </c>
       <c r="E14" s="27" t="n">
         <v>498866214</v>
@@ -2031,7 +2030,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>583256268</v>
+        <v>543282274</v>
       </c>
       <c r="E15" s="27" t="n">
         <v>119727891</v>
@@ -2071,7 +2070,7 @@
         </is>
       </c>
       <c r="D16" s="27" t="n">
-        <v>1161621042</v>
+        <v>1230123482</v>
       </c>
       <c r="E16" s="27" t="n">
         <v>399092971</v>
@@ -2234,7 +2233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F166"/>
+  <dimension ref="A1:F163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2252,7 +2251,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="24" t="inlineStr">
         <is>
@@ -2468,7 +2466,6 @@
         <v>2270422</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="36" t="inlineStr">
         <is>
@@ -2512,7 +2509,6 @@
         <v>2270422</v>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="36" t="inlineStr">
         <is>
@@ -2724,7 +2720,6 @@
         <v>2270422</v>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="36" t="inlineStr">
         <is>
@@ -2824,7 +2819,6 @@
         <v>26894000</v>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="36" t="inlineStr">
         <is>
@@ -3788,7 +3782,6 @@
         <v>1710740</v>
       </c>
     </row>
-    <row r="64"/>
     <row r="65">
       <c r="A65" s="36" t="inlineStr">
         <is>
@@ -5148,7 +5141,6 @@
         <v>1710740</v>
       </c>
     </row>
-    <row r="114"/>
     <row r="115">
       <c r="A115" s="36" t="inlineStr">
         <is>
@@ -6226,7 +6218,6 @@
         <v>2270422</v>
       </c>
     </row>
-    <row r="155"/>
     <row r="156">
       <c r="A156" s="36" t="inlineStr">
         <is>
@@ -6270,7 +6261,6 @@
         <v>11234100</v>
       </c>
     </row>
-    <row r="158"/>
     <row r="159">
       <c r="A159" s="36" t="inlineStr">
         <is>
@@ -6342,6 +6332,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="162"/>
     <row r="163">
       <c r="A163" s="49" t="inlineStr">
         <is>
@@ -6352,9 +6343,6 @@
         <v>372666880</v>
       </c>
     </row>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A159:D159"/>
@@ -6768,7 +6756,7 @@
       </c>
       <c r="B5" s="61" t="inlineStr">
         <is>
-          <t>9/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(bhx): nang tong CH BHX len 240, ap dung cong thuc 5 hub/240 va cap nhat so CH BHX 11 NV (v1.3.3 - Code 34)
</commit_message>
<xml_diff>
--- a/Team_CamGiang_Report.xlsx
+++ b/Team_CamGiang_Report.xlsx
@@ -1200,19 +1200,19 @@
         <v>12299713233</v>
       </c>
       <c r="B7" s="12" t="n">
-        <v>3911111125</v>
+        <v>3838609228</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>359247028</v>
       </c>
       <c r="D7" s="12" t="n">
-        <v>4270358153</v>
+        <v>4197856256</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>7563511176</v>
+        <v>8101856977</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.360858991617821</v>
+        <v>0.3412970836374621</v>
       </c>
       <c r="G7" s="14" t="n">
         <v>0.3612647089323572</v>
@@ -1282,16 +1282,16 @@
         <v>1427158977</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>498866214</v>
+        <v>462947847</v>
       </c>
       <c r="F13" s="19" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>498866214</v>
+        <v>462947847</v>
       </c>
       <c r="H13" s="20" t="n">
-        <v>0.3704934749118172</v>
+        <v>0.3243842167977338</v>
       </c>
     </row>
     <row r="14">
@@ -1307,16 +1307,16 @@
         <v>1490030916</v>
       </c>
       <c r="E14" s="19" t="n">
-        <v>478911565</v>
+        <v>501526834</v>
       </c>
       <c r="F14" s="19" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="19" t="n">
-        <v>478911565</v>
+        <v>501526834</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>0.370493474537032</v>
+        <v>0.3365882067375842</v>
       </c>
     </row>
     <row r="15">
@@ -1332,16 +1332,16 @@
         <v>1553803206</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>498866214</v>
+        <v>520816327</v>
       </c>
       <c r="F15" s="19" t="n">
         <v>2270422</v>
       </c>
       <c r="G15" s="19" t="n">
-        <v>501136636</v>
+        <v>523086749</v>
       </c>
       <c r="H15" s="20" t="n">
-        <v>0.3698841468044531</v>
+        <v>0.3366492918666304</v>
       </c>
     </row>
     <row r="16">
@@ -1357,16 +1357,16 @@
         <v>1439209643</v>
       </c>
       <c r="E16" s="19" t="n">
-        <v>498866214</v>
+        <v>462947847</v>
       </c>
       <c r="F16" s="19" t="n">
         <v>15438632</v>
       </c>
       <c r="G16" s="19" t="n">
-        <v>514304846</v>
+        <v>478386479</v>
       </c>
       <c r="H16" s="20" t="n">
-        <v>0.367491941705772</v>
+        <v>0.3323952707840493</v>
       </c>
     </row>
     <row r="17">
@@ -1382,16 +1382,16 @@
         <v>1224747376</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>419047620</v>
+        <v>405079366</v>
       </c>
       <c r="F17" s="19" t="n">
         <v>13622532</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>432670152</v>
+        <v>418701898</v>
       </c>
       <c r="H17" s="20" t="n">
-        <v>0.3663000112107219</v>
+        <v>0.3418679690235156</v>
       </c>
     </row>
     <row r="18">
@@ -1407,16 +1407,16 @@
         <v>1347067397</v>
       </c>
       <c r="E18" s="19" t="n">
-        <v>419047620</v>
+        <v>424368859</v>
       </c>
       <c r="F18" s="19" t="n">
         <v>34581126</v>
       </c>
       <c r="G18" s="19" t="n">
-        <v>453628746</v>
+        <v>458949985</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>0.3655489147090821</v>
+        <v>0.3407030606056602</v>
       </c>
     </row>
     <row r="19">
@@ -1432,16 +1432,16 @@
         <v>543282274</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>119727891</v>
+        <v>115736962</v>
       </c>
       <c r="F19" s="19" t="n">
         <v>88421641</v>
       </c>
       <c r="G19" s="19" t="n">
-        <v>208149532</v>
+        <v>204158603</v>
       </c>
       <c r="H19" s="20" t="n">
-        <v>0.3568749166018392</v>
+        <v>0.3757873443888581</v>
       </c>
     </row>
     <row r="20">
@@ -1457,16 +1457,16 @@
         <v>1230123482</v>
       </c>
       <c r="E20" s="19" t="n">
-        <v>399092971</v>
+        <v>385789872</v>
       </c>
       <c r="F20" s="19" t="n">
         <v>11234100</v>
       </c>
       <c r="G20" s="19" t="n">
-        <v>410327071</v>
+        <v>397023972</v>
       </c>
       <c r="H20" s="20" t="n">
-        <v>0.3532366031296461</v>
+        <v>0.3227513154650924</v>
       </c>
     </row>
     <row r="21">
@@ -1482,16 +1482,16 @@
         <v>735943613</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>219501134</v>
+        <v>212184430</v>
       </c>
       <c r="F21" s="19" t="n">
         <v>79239773</v>
       </c>
       <c r="G21" s="19" t="n">
-        <v>298740907</v>
+        <v>291424203</v>
       </c>
       <c r="H21" s="20" t="n">
-        <v>0.3454404477334937</v>
+        <v>0.3959871352263505</v>
       </c>
     </row>
     <row r="22">
@@ -1516,7 +1516,7 @@
         <v>114438802</v>
       </c>
       <c r="H22" s="20" t="n">
-        <v>0.2853565874090838</v>
+        <v>0.3804269621968423</v>
       </c>
     </row>
     <row r="23">
@@ -1532,16 +1532,16 @@
         <v>1007529600</v>
       </c>
       <c r="E23" s="19" t="n">
-        <v>359183682</v>
+        <v>347210885</v>
       </c>
       <c r="F23" s="19" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="19" t="n">
-        <v>359183682</v>
+        <v>347210885</v>
       </c>
       <c r="H23" s="20" t="n">
-        <v>0.3564993842364532</v>
+        <v>0.3446160638853688</v>
       </c>
     </row>
   </sheetData>
@@ -1607,18 +1607,15 @@
       <c r="C3" s="22" t="n">
         <v>0.4667</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Tổng CH BHX:</t>
-        </is>
+      <c r="E3" s="2" t="n">
+        <v>240</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>232</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>TB BHX/CH:</t>
-        </is>
+      <c r="H3" s="2">
+        <f>'Data BHX'!B5</f>
+        <v/>
       </c>
       <c r="I3" s="23" t="n">
         <v>19954649</v>
@@ -1712,8 +1709,9 @@
       <c r="D7" s="27" t="n">
         <v>1224747376</v>
       </c>
-      <c r="E7" s="27" t="n">
-        <v>419047620</v>
+      <c r="E7" s="27">
+        <f>'Data BHX'!E8</f>
+        <v/>
       </c>
       <c r="F7" s="27" t="n">
         <v>13622532</v>
@@ -1752,8 +1750,9 @@
       <c r="D8" s="27" t="n">
         <v>1553803206</v>
       </c>
-      <c r="E8" s="27" t="n">
-        <v>498866214</v>
+      <c r="E8" s="27">
+        <f>'Data BHX'!E9</f>
+        <v/>
       </c>
       <c r="F8" s="27" t="n">
         <v>2270422</v>
@@ -1792,8 +1791,9 @@
       <c r="D9" s="27" t="n">
         <v>1439209643</v>
       </c>
-      <c r="E9" s="27" t="n">
-        <v>498866214</v>
+      <c r="E9" s="27">
+        <f>'Data BHX'!E10</f>
+        <v/>
       </c>
       <c r="F9" s="27" t="n">
         <v>13622532</v>
@@ -1832,8 +1832,9 @@
       <c r="D10" s="27" t="n">
         <v>1347067397</v>
       </c>
-      <c r="E10" s="27" t="n">
-        <v>419047620</v>
+      <c r="E10" s="27">
+        <f>'Data BHX'!E11</f>
+        <v/>
       </c>
       <c r="F10" s="27" t="n">
         <v>0</v>
@@ -1872,8 +1873,9 @@
       <c r="D11" s="27" t="n">
         <v>1490030916</v>
       </c>
-      <c r="E11" s="27" t="n">
-        <v>478911565</v>
+      <c r="E11" s="27">
+        <f>'Data BHX'!E12</f>
+        <v/>
       </c>
       <c r="F11" s="27" t="n">
         <v>0</v>
@@ -1912,8 +1914,9 @@
       <c r="D12" s="27" t="n">
         <v>735943613</v>
       </c>
-      <c r="E12" s="27" t="n">
-        <v>219501134</v>
+      <c r="E12" s="27">
+        <f>'Data BHX'!E13</f>
+        <v/>
       </c>
       <c r="F12" s="27" t="n">
         <v>54490128</v>
@@ -1952,8 +1955,9 @@
       <c r="D13" s="27" t="n">
         <v>300816749</v>
       </c>
-      <c r="E13" s="27" t="n">
-        <v>0</v>
+      <c r="E13" s="27">
+        <f>'Data BHX'!E14</f>
+        <v/>
       </c>
       <c r="F13" s="27" t="n">
         <v>45408440</v>
@@ -1992,8 +1996,9 @@
       <c r="D14" s="27" t="n">
         <v>1427158977</v>
       </c>
-      <c r="E14" s="27" t="n">
-        <v>498866214</v>
+      <c r="E14" s="27">
+        <f>'Data BHX'!E15</f>
+        <v/>
       </c>
       <c r="F14" s="27" t="n">
         <v>0</v>
@@ -2032,8 +2037,9 @@
       <c r="D15" s="27" t="n">
         <v>543282274</v>
       </c>
-      <c r="E15" s="27" t="n">
-        <v>119727891</v>
+      <c r="E15" s="27">
+        <f>'Data BHX'!E16</f>
+        <v/>
       </c>
       <c r="F15" s="27" t="n">
         <v>29515486</v>
@@ -2072,8 +2078,9 @@
       <c r="D16" s="27" t="n">
         <v>1230123482</v>
       </c>
-      <c r="E16" s="27" t="n">
-        <v>399092971</v>
+      <c r="E16" s="27">
+        <f>'Data BHX'!E17</f>
+        <v/>
       </c>
       <c r="F16" s="27" t="n">
         <v>0</v>
@@ -2112,8 +2119,9 @@
       <c r="D17" s="27" t="n">
         <v>1007529600</v>
       </c>
-      <c r="E17" s="27" t="n">
-        <v>359183682</v>
+      <c r="E17" s="27">
+        <f>'Data BHX'!E18</f>
+        <v/>
       </c>
       <c r="F17" s="27" t="n">
         <v>0</v>
@@ -6366,7 +6374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6380,7 +6388,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="51" t="inlineStr">
         <is>
-          <t>PHÂN BỔ DOANH SỐ BHX (232 CỬA HÀNG)</t>
+          <t>PHÂN BỔ DOANH SỐ BHX (240 CỬA HÀNG)</t>
         </is>
       </c>
     </row>
@@ -6401,7 +6409,7 @@
         </is>
       </c>
       <c r="B4" s="53" t="n">
-        <v>232</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5">
@@ -6463,11 +6471,13 @@
         <f>$B$5</f>
         <v/>
       </c>
-      <c r="E8" s="55" t="n">
-        <v>419047620</v>
-      </c>
-      <c r="F8" s="56" t="n">
-        <v>0.09051724137931035</v>
+      <c r="E8" s="55">
+        <f>C8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="56">
+        <f>E8/$E$19</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -6480,17 +6490,19 @@
         </is>
       </c>
       <c r="C9" s="26" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D9" s="55">
         <f>$B$5</f>
         <v/>
       </c>
-      <c r="E9" s="55" t="n">
-        <v>498866214</v>
-      </c>
-      <c r="F9" s="56" t="n">
-        <v>0.1077586206896552</v>
+      <c r="E9" s="55">
+        <f>C9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="56">
+        <f>E9/$E$19</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -6503,17 +6515,19 @@
         </is>
       </c>
       <c r="C10" s="26" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D10" s="55">
         <f>$B$5</f>
         <v/>
       </c>
-      <c r="E10" s="55" t="n">
-        <v>498866214</v>
-      </c>
-      <c r="F10" s="56" t="n">
-        <v>0.1077586206896552</v>
+      <c r="E10" s="55">
+        <f>C10*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="56">
+        <f>E10/$E$19</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -6526,17 +6540,19 @@
         </is>
       </c>
       <c r="C11" s="26" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D11" s="55">
         <f>$B$5</f>
         <v/>
       </c>
-      <c r="E11" s="55" t="n">
-        <v>419047620</v>
-      </c>
-      <c r="F11" s="56" t="n">
-        <v>0.09051724137931035</v>
+      <c r="E11" s="55">
+        <f>C11*D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="56">
+        <f>E11/$E$19</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -6549,17 +6565,19 @@
         </is>
       </c>
       <c r="C12" s="26" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D12" s="55">
         <f>$B$5</f>
         <v/>
       </c>
-      <c r="E12" s="55" t="n">
-        <v>478911565</v>
-      </c>
-      <c r="F12" s="56" t="n">
-        <v>0.103448275862069</v>
+      <c r="E12" s="55">
+        <f>C12*D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="56">
+        <f>E12/$E$19</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -6578,11 +6596,13 @@
         <f>$B$5</f>
         <v/>
       </c>
-      <c r="E13" s="55" t="n">
-        <v>219501134</v>
-      </c>
-      <c r="F13" s="56" t="n">
-        <v>0.04741379310344827</v>
+      <c r="E13" s="55">
+        <f>C13*D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="56">
+        <f>E13/$E$19</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -6601,11 +6621,13 @@
         <f>$B$5</f>
         <v/>
       </c>
-      <c r="E14" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="56" t="n">
-        <v>0</v>
+      <c r="E14" s="55">
+        <f>C14*D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="56">
+        <f>E14/$E$19</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -6618,17 +6640,19 @@
         </is>
       </c>
       <c r="C15" s="26" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D15" s="55">
         <f>$B$5</f>
         <v/>
       </c>
-      <c r="E15" s="55" t="n">
-        <v>498866214</v>
-      </c>
-      <c r="F15" s="56" t="n">
-        <v>0.1077586206896552</v>
+      <c r="E15" s="55">
+        <f>C15*D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="56">
+        <f>E15/$E$19</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -6647,11 +6671,13 @@
         <f>$B$5</f>
         <v/>
       </c>
-      <c r="E16" s="55" t="n">
-        <v>119727891</v>
-      </c>
-      <c r="F16" s="56" t="n">
-        <v>0.02586206896551724</v>
+      <c r="E16" s="55">
+        <f>C16*D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="56">
+        <f>E16/$E$19</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -6670,30 +6696,59 @@
         <f>$B$5</f>
         <v/>
       </c>
-      <c r="E17" s="55" t="n">
-        <v>399092971</v>
-      </c>
-      <c r="F17" s="56" t="n">
-        <v>0.08620689655172414</v>
+      <c r="E17" s="55">
+        <f>C17*D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="56">
+        <f>E17/$E$19</f>
+        <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="30" t="inlineStr"/>
-      <c r="B18" s="57" t="inlineStr">
+      <c r="A18" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Võ Thị Hằng</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="n">
+        <v>18</v>
+      </c>
+      <c r="D18" s="55">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E18" s="55">
+        <f>C18*D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="56">
+        <f>E18/$E$19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr"/>
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>TỔNG</t>
         </is>
       </c>
-      <c r="C18" s="58" t="n">
-        <v>178</v>
-      </c>
-      <c r="D18" s="30" t="n"/>
-      <c r="E18" s="59">
-        <f>SUM(E8:E17)</f>
-        <v/>
-      </c>
-      <c r="F18" s="60" t="n">
-        <v>0.7672413793103449</v>
+      <c r="C19" s="26">
+        <f>SUM(C8:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="55" t="n"/>
+      <c r="E19" s="55">
+        <f>SUM(E8:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="56">
+        <f>E19/$B$3</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -6803,7 +6858,7 @@
         </is>
       </c>
       <c r="B9" s="61" t="n">
-        <v>232</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10">

</xml_diff>